<commit_message>
Rewrite of summary tables
</commit_message>
<xml_diff>
--- a/output/Europe_summary.xlsx
+++ b/output/Europe_summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve">country_code</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t xml:space="preserve">SK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UK</t>
   </si>
 </sst>
 </file>
@@ -479,21 +482,21 @@
         <v>8</v>
       </c>
       <c r="B2" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C2" t="n">
-        <v>4920</v>
+        <v>4084</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="n">
-        <v>4918</v>
+        <v>4085</v>
       </c>
       <c r="F2" t="n">
-        <v>35410530</v>
+        <v>25562436</v>
       </c>
       <c r="G2"/>
       <c r="H2" t="n">
-        <v>35383912</v>
+        <v>25562000</v>
       </c>
     </row>
     <row r="3">
@@ -501,21 +504,21 @@
         <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C3" t="n">
-        <v>18875</v>
+        <v>4250</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="n">
-        <v>4719</v>
+        <v>4242</v>
       </c>
       <c r="F3" t="n">
-        <v>150539587</v>
+        <v>29654490</v>
       </c>
       <c r="G3"/>
       <c r="H3" t="n">
-        <v>37634895</v>
+        <v>29595797</v>
       </c>
     </row>
     <row r="4">
@@ -523,21 +526,21 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C4" t="n">
-        <v>20681</v>
+        <v>9054</v>
       </c>
       <c r="D4"/>
       <c r="E4" t="n">
-        <v>5170</v>
+        <v>4497</v>
       </c>
       <c r="F4" t="n">
-        <v>176872366</v>
+        <v>62412061</v>
       </c>
       <c r="G4"/>
       <c r="H4" t="n">
-        <v>44218080</v>
+        <v>30152193</v>
       </c>
     </row>
     <row r="5">
@@ -545,2052 +548,3976 @@
         <v>8</v>
       </c>
       <c r="B5" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C5" t="n">
-        <v>20031</v>
+        <v>4920</v>
       </c>
       <c r="D5"/>
-      <c r="E5"/>
+      <c r="E5" t="n">
+        <v>4918</v>
+      </c>
       <c r="F5" t="n">
-        <v>162044148</v>
+        <v>35410530</v>
       </c>
       <c r="G5"/>
-      <c r="H5"/>
+      <c r="H5" t="n">
+        <v>35383912</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C6" t="n">
-        <v>223</v>
-      </c>
-      <c r="D6" t="n">
-        <v>223</v>
-      </c>
+        <v>18875</v>
+      </c>
+      <c r="D6"/>
       <c r="E6" t="n">
-        <v>223</v>
+        <v>4719</v>
       </c>
       <c r="F6" t="n">
-        <v>1447493</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1446425</v>
-      </c>
+        <v>150539587</v>
+      </c>
+      <c r="G6"/>
       <c r="H6" t="n">
-        <v>1447320</v>
+        <v>37634895</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C7" t="n">
-        <v>243</v>
-      </c>
-      <c r="D7" t="n">
-        <v>243</v>
-      </c>
+        <v>20681</v>
+      </c>
+      <c r="D7"/>
       <c r="E7" t="n">
-        <v>243</v>
+        <v>5170</v>
       </c>
       <c r="F7" t="n">
-        <v>1738908</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1740569</v>
-      </c>
+        <v>176872366</v>
+      </c>
+      <c r="G7"/>
       <c r="H7" t="n">
-        <v>1739960</v>
+        <v>44218080</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C8" t="n">
-        <v>261</v>
-      </c>
-      <c r="D8" t="n">
-        <v>261</v>
-      </c>
-      <c r="E8" t="n">
-        <v>261</v>
-      </c>
+        <v>20031</v>
+      </c>
+      <c r="D8"/>
+      <c r="E8"/>
       <c r="F8" t="n">
-        <v>2145942</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1822632</v>
-      </c>
-      <c r="H8" t="n">
-        <v>1832170</v>
-      </c>
+        <v>162044148</v>
+      </c>
+      <c r="G8"/>
+      <c r="H8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C9" t="n">
-        <v>42904</v>
-      </c>
-      <c r="D9"/>
+        <v>111</v>
+      </c>
+      <c r="D9" t="n">
+        <v>111</v>
+      </c>
       <c r="E9" t="n">
-        <v>10726</v>
+        <v>111</v>
       </c>
       <c r="F9" t="n">
-        <v>121418152</v>
-      </c>
-      <c r="G9"/>
+        <v>841047</v>
+      </c>
+      <c r="G9" t="n">
+        <v>844587</v>
+      </c>
       <c r="H9" t="n">
-        <v>30354537</v>
+        <v>841000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C10" t="n">
-        <v>36255</v>
-      </c>
-      <c r="D10"/>
+        <v>86</v>
+      </c>
+      <c r="D10" t="n">
+        <v>86</v>
+      </c>
       <c r="E10" t="n">
-        <v>9064</v>
+        <v>86</v>
       </c>
       <c r="F10" t="n">
-        <v>123199484</v>
-      </c>
-      <c r="G10"/>
+        <v>538016</v>
+      </c>
+      <c r="G10" t="n">
+        <v>536385</v>
+      </c>
       <c r="H10" t="n">
-        <v>30799871</v>
+        <v>538347</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C11" t="n">
-        <v>39713</v>
-      </c>
-      <c r="D11"/>
+        <v>209</v>
+      </c>
+      <c r="D11" t="n">
+        <v>209</v>
+      </c>
       <c r="E11" t="n">
-        <v>9928</v>
+        <v>209</v>
       </c>
       <c r="F11" t="n">
-        <v>163358968</v>
-      </c>
-      <c r="G11"/>
+        <v>1394030</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1401185</v>
+      </c>
       <c r="H11" t="n">
-        <v>40839740</v>
+        <v>1394030</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B12" t="n">
         <v>2021</v>
       </c>
       <c r="C12" t="n">
-        <v>31449</v>
-      </c>
-      <c r="D12"/>
+        <v>223</v>
+      </c>
+      <c r="D12" t="n">
+        <v>223</v>
+      </c>
       <c r="E12" t="n">
-        <v>7862</v>
+        <v>223</v>
       </c>
       <c r="F12" t="n">
-        <v>180210643</v>
-      </c>
-      <c r="G12"/>
+        <v>1447493</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1446425</v>
+      </c>
       <c r="H12" t="n">
-        <v>45052661</v>
+        <v>1447320</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13" t="n">
         <v>2022</v>
       </c>
       <c r="C13" t="n">
-        <v>30376</v>
-      </c>
-      <c r="D13"/>
+        <v>243</v>
+      </c>
+      <c r="D13" t="n">
+        <v>243</v>
+      </c>
       <c r="E13" t="n">
-        <v>7594</v>
+        <v>243</v>
       </c>
       <c r="F13" t="n">
-        <v>191747022</v>
-      </c>
-      <c r="G13"/>
+        <v>1738908</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1740569</v>
+      </c>
       <c r="H13" t="n">
-        <v>47936756</v>
+        <v>1739960</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B14" t="n">
         <v>2023</v>
       </c>
       <c r="C14" t="n">
-        <v>22801</v>
-      </c>
-      <c r="D14"/>
+        <v>261</v>
+      </c>
+      <c r="D14" t="n">
+        <v>261</v>
+      </c>
       <c r="E14" t="n">
-        <v>5700</v>
+        <v>261</v>
       </c>
       <c r="F14" t="n">
-        <v>156446683</v>
-      </c>
-      <c r="G14"/>
+        <v>2145942</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1822632</v>
+      </c>
       <c r="H14" t="n">
-        <v>39111670</v>
+        <v>1832170</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B15" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C15" t="n">
-        <v>83964</v>
+        <v>43034</v>
       </c>
       <c r="D15"/>
       <c r="E15" t="n">
-        <v>20991</v>
+        <v>10757</v>
       </c>
       <c r="F15" t="n">
-        <v>178246786</v>
+        <v>117533075</v>
       </c>
       <c r="G15"/>
       <c r="H15" t="n">
-        <v>44561696</v>
+        <v>29386000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B16" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C16" t="n">
-        <v>77036</v>
+        <v>47838</v>
       </c>
       <c r="D16"/>
       <c r="E16" t="n">
-        <v>19259</v>
+        <v>11963</v>
       </c>
       <c r="F16" t="n">
-        <v>196879839</v>
+        <v>118704297</v>
       </c>
       <c r="G16"/>
       <c r="H16" t="n">
-        <v>49219960</v>
+        <v>29718882</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B17" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C17" t="n">
-        <v>74453</v>
+        <v>35440</v>
       </c>
       <c r="D17"/>
       <c r="E17" t="n">
-        <v>18613</v>
+        <v>8863</v>
       </c>
       <c r="F17" t="n">
-        <v>202467102</v>
+        <v>96988930</v>
       </c>
       <c r="G17"/>
       <c r="H17" t="n">
-        <v>50616780</v>
+        <v>24280249</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B18" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C18" t="n">
-        <v>74740</v>
+        <v>42904</v>
       </c>
       <c r="D18"/>
-      <c r="E18"/>
+      <c r="E18" t="n">
+        <v>10726</v>
+      </c>
       <c r="F18" t="n">
-        <v>204685557</v>
+        <v>121418152</v>
       </c>
       <c r="G18"/>
-      <c r="H18"/>
+      <c r="H18" t="n">
+        <v>30354537</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B19" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C19" t="n">
-        <v>48977</v>
+        <v>36255</v>
       </c>
       <c r="D19"/>
       <c r="E19" t="n">
-        <v>32165</v>
+        <v>9064</v>
       </c>
       <c r="F19" t="n">
-        <v>186471144</v>
+        <v>123199484</v>
       </c>
       <c r="G19"/>
       <c r="H19" t="n">
-        <v>121852712</v>
+        <v>30799871</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B20" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C20" t="n">
-        <v>40229</v>
+        <v>39713</v>
       </c>
       <c r="D20"/>
       <c r="E20" t="n">
-        <v>26692</v>
+        <v>9928</v>
       </c>
       <c r="F20" t="n">
-        <v>179085773</v>
+        <v>163358968</v>
       </c>
       <c r="G20"/>
       <c r="H20" t="n">
-        <v>111365503</v>
+        <v>40839740</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B21" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="C21" t="n">
-        <v>56035</v>
+        <v>29388</v>
       </c>
       <c r="D21"/>
       <c r="E21" t="n">
-        <v>35230</v>
+        <v>7347</v>
       </c>
       <c r="F21" t="n">
-        <v>205951493</v>
+        <v>156003834</v>
       </c>
       <c r="G21"/>
       <c r="H21" t="n">
-        <v>133123810</v>
+        <v>39001000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B22" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C22" t="n">
-        <v>142559</v>
+        <v>32316</v>
       </c>
       <c r="D22"/>
       <c r="E22" t="n">
-        <v>37308</v>
+        <v>8079</v>
       </c>
       <c r="F22" t="n">
-        <v>431222582</v>
+        <v>175011200</v>
       </c>
       <c r="G22"/>
       <c r="H22" t="n">
-        <v>123721340</v>
+        <v>43752800</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B23" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C23" t="n">
-        <v>144802</v>
+        <v>29371</v>
       </c>
       <c r="D23"/>
       <c r="E23" t="n">
-        <v>39617</v>
+        <v>7343</v>
       </c>
       <c r="F23" t="n">
-        <v>455587353</v>
+        <v>148074343</v>
       </c>
       <c r="G23"/>
       <c r="H23" t="n">
-        <v>142325671</v>
+        <v>37023565</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B24" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C24" t="n">
-        <v>121956</v>
+        <v>31449</v>
       </c>
       <c r="D24"/>
       <c r="E24" t="n">
-        <v>23207</v>
+        <v>7862</v>
       </c>
       <c r="F24" t="n">
-        <v>404838537</v>
+        <v>180210643</v>
       </c>
       <c r="G24"/>
       <c r="H24" t="n">
-        <v>101209630</v>
+        <v>45052661</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B25" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C25" t="n">
-        <v>1882</v>
+        <v>30376</v>
       </c>
       <c r="D25"/>
       <c r="E25" t="n">
-        <v>849</v>
+        <v>7594</v>
       </c>
       <c r="F25" t="n">
-        <v>9178512</v>
+        <v>191747022</v>
       </c>
       <c r="G25"/>
       <c r="H25" t="n">
-        <v>4323241</v>
+        <v>47936756</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B26" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C26" t="n">
-        <v>1969</v>
+        <v>22801</v>
       </c>
       <c r="D26"/>
       <c r="E26" t="n">
-        <v>807</v>
+        <v>5700</v>
       </c>
       <c r="F26" t="n">
-        <v>10627352</v>
+        <v>156446683</v>
       </c>
       <c r="G26"/>
       <c r="H26" t="n">
-        <v>4928630</v>
+        <v>39111670</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B27" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="C27" t="n">
-        <v>2104</v>
+        <v>87000</v>
       </c>
       <c r="D27"/>
       <c r="E27" t="n">
-        <v>921</v>
+        <v>21750</v>
       </c>
       <c r="F27" t="n">
-        <v>11964815</v>
+        <v>194380004</v>
       </c>
       <c r="G27"/>
       <c r="H27" t="n">
-        <v>5737970</v>
+        <v>48595000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B28" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C28" t="n">
-        <v>574777</v>
+        <v>83956</v>
       </c>
       <c r="D28"/>
       <c r="E28" t="n">
-        <v>143694</v>
+        <v>20989</v>
       </c>
       <c r="F28" t="n">
-        <v>2563437015</v>
+        <v>164947094</v>
       </c>
       <c r="G28"/>
       <c r="H28" t="n">
-        <v>640859254</v>
+        <v>41236773</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B29" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C29" t="n">
-        <v>561809</v>
+        <v>81608</v>
       </c>
       <c r="D29"/>
       <c r="E29" t="n">
-        <v>141333</v>
+        <v>20612</v>
       </c>
       <c r="F29" t="n">
-        <v>3379295345</v>
+        <v>155772139</v>
       </c>
       <c r="G29"/>
       <c r="H29" t="n">
-        <v>851690964</v>
+        <v>39378702</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B30" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C30" t="n">
-        <v>563631</v>
+        <v>83964</v>
       </c>
       <c r="D30"/>
       <c r="E30" t="n">
-        <v>140908</v>
+        <v>20991</v>
       </c>
       <c r="F30" t="n">
-        <v>2735223696</v>
+        <v>178246786</v>
       </c>
       <c r="G30"/>
       <c r="H30" t="n">
-        <v>683805930</v>
+        <v>44561696</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B31" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C31" t="n">
-        <v>1106259</v>
+        <v>77036</v>
       </c>
       <c r="D31"/>
       <c r="E31" t="n">
-        <v>276565</v>
+        <v>19259</v>
       </c>
       <c r="F31" t="n">
-        <v>2594433985</v>
+        <v>196879839</v>
       </c>
       <c r="G31"/>
       <c r="H31" t="n">
-        <v>648608496</v>
+        <v>49219960</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B32" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C32" t="n">
-        <v>1090359</v>
+        <v>74453</v>
       </c>
       <c r="D32"/>
       <c r="E32" t="n">
-        <v>272990</v>
+        <v>18613</v>
       </c>
       <c r="F32" t="n">
-        <v>3214508553</v>
+        <v>202467102</v>
       </c>
       <c r="G32"/>
       <c r="H32" t="n">
-        <v>808727377</v>
+        <v>50616780</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B33" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C33" t="n">
-        <v>971014</v>
+        <v>74740</v>
       </c>
       <c r="D33"/>
-      <c r="E33" t="n">
-        <v>242754</v>
-      </c>
+      <c r="E33"/>
       <c r="F33" t="n">
-        <v>3206663423</v>
+        <v>204685557</v>
       </c>
       <c r="G33"/>
-      <c r="H33" t="n">
-        <v>801665850</v>
-      </c>
+      <c r="H33"/>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B34" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C34" t="n">
-        <v>57598</v>
+        <v>56435</v>
       </c>
       <c r="D34"/>
       <c r="E34" t="n">
-        <v>14399</v>
+        <v>33090</v>
       </c>
       <c r="F34" t="n">
-        <v>262937076</v>
+        <v>156163205</v>
       </c>
       <c r="G34"/>
       <c r="H34" t="n">
-        <v>65734269</v>
+        <v>112572000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B35" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C35" t="n">
-        <v>65122</v>
+        <v>72627</v>
       </c>
       <c r="D35"/>
       <c r="E35" t="n">
-        <v>16280</v>
+        <v>41077</v>
       </c>
       <c r="F35" t="n">
-        <v>373857804</v>
+        <v>191053851</v>
       </c>
       <c r="G35"/>
       <c r="H35" t="n">
-        <v>93464451</v>
+        <v>126108719</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B36" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C36" t="n">
-        <v>60674</v>
+        <v>52375</v>
       </c>
       <c r="D36"/>
       <c r="E36" t="n">
-        <v>15168</v>
+        <v>32397</v>
       </c>
       <c r="F36" t="n">
-        <v>341522340</v>
+        <v>193135578</v>
       </c>
       <c r="G36"/>
       <c r="H36" t="n">
-        <v>85380590</v>
+        <v>121091683</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B37" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C37" t="n">
-        <v>66465</v>
+        <v>48977</v>
       </c>
       <c r="D37"/>
-      <c r="E37"/>
+      <c r="E37" t="n">
+        <v>32165</v>
+      </c>
       <c r="F37" t="n">
-        <v>346245538</v>
+        <v>186471144</v>
       </c>
       <c r="G37"/>
-      <c r="H37"/>
+      <c r="H37" t="n">
+        <v>121852712</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B38" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C38" t="n">
-        <v>773576</v>
+        <v>40229</v>
       </c>
       <c r="D38"/>
       <c r="E38" t="n">
-        <v>193394</v>
+        <v>26692</v>
       </c>
       <c r="F38" t="n">
-        <v>3124134782</v>
+        <v>179085773</v>
       </c>
       <c r="G38"/>
       <c r="H38" t="n">
-        <v>781033695</v>
+        <v>111365503</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B39" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C39" t="n">
-        <v>736208</v>
+        <v>56035</v>
       </c>
       <c r="D39"/>
       <c r="E39" t="n">
-        <v>184052</v>
+        <v>35230</v>
       </c>
       <c r="F39" t="n">
-        <v>3166130132</v>
+        <v>205951493</v>
       </c>
       <c r="G39"/>
       <c r="H39" t="n">
-        <v>791532532</v>
+        <v>133123810</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B40" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="C40" t="n">
-        <v>746246</v>
+        <v>128667</v>
       </c>
       <c r="D40"/>
       <c r="E40" t="n">
-        <v>186562</v>
+        <v>33195</v>
       </c>
       <c r="F40" t="n">
-        <v>3622938207</v>
+        <v>127111451</v>
       </c>
       <c r="G40"/>
       <c r="H40" t="n">
-        <v>905734580</v>
+        <v>110115000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B41" t="n">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="C41" t="n">
-        <v>725737</v>
+        <v>160886</v>
       </c>
       <c r="D41"/>
-      <c r="E41"/>
+      <c r="E41" t="n">
+        <v>40221</v>
+      </c>
       <c r="F41" t="n">
-        <v>3428948717</v>
+        <v>243009955</v>
       </c>
       <c r="G41"/>
-      <c r="H41"/>
+      <c r="H41" t="n">
+        <v>124463826</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B42" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C42" t="n">
-        <v>123190</v>
-      </c>
-      <c r="D42" t="n">
-        <v>27920</v>
-      </c>
+        <v>151357</v>
+      </c>
+      <c r="D42"/>
       <c r="E42" t="n">
-        <v>26831</v>
+        <v>41185</v>
       </c>
       <c r="F42" t="n">
-        <v>694026961</v>
-      </c>
-      <c r="G42" t="n">
-        <v>167033674</v>
-      </c>
+        <v>222474240</v>
+      </c>
+      <c r="G42"/>
       <c r="H42" t="n">
-        <v>162243534</v>
+        <v>121216657</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B43" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C43" t="n">
-        <v>120127</v>
-      </c>
-      <c r="D43" t="n">
-        <v>27218</v>
-      </c>
+        <v>142559</v>
+      </c>
+      <c r="D43"/>
       <c r="E43" t="n">
-        <v>27197</v>
+        <v>37308</v>
       </c>
       <c r="F43" t="n">
-        <v>740738278</v>
-      </c>
-      <c r="G43" t="n">
-        <v>177813277</v>
-      </c>
+        <v>431222582</v>
+      </c>
+      <c r="G43"/>
       <c r="H43" t="n">
-        <v>177097530</v>
+        <v>123721340</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B44" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C44" t="n">
-        <v>84254</v>
-      </c>
-      <c r="D44" t="n">
-        <v>26824</v>
-      </c>
+        <v>144802</v>
+      </c>
+      <c r="D44"/>
       <c r="E44" t="n">
-        <v>26859</v>
+        <v>39617</v>
       </c>
       <c r="F44" t="n">
-        <v>625028160</v>
-      </c>
-      <c r="G44" t="n">
-        <v>202702558</v>
-      </c>
+        <v>455587353</v>
+      </c>
+      <c r="G44"/>
       <c r="H44" t="n">
-        <v>203839780</v>
+        <v>142325671</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B45" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C45" t="n">
-        <v>90884</v>
+        <v>121956</v>
       </c>
       <c r="D45"/>
-      <c r="E45"/>
+      <c r="E45" t="n">
+        <v>23207</v>
+      </c>
       <c r="F45" t="n">
-        <v>595783690</v>
+        <v>404838537</v>
       </c>
       <c r="G45"/>
-      <c r="H45"/>
+      <c r="H45" t="n">
+        <v>101209630</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B46" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C46" t="n">
-        <v>71823</v>
-      </c>
-      <c r="D46" t="n">
-        <v>18025</v>
-      </c>
+        <v>1244</v>
+      </c>
+      <c r="D46"/>
       <c r="E46" t="n">
-        <v>17956</v>
+        <v>944</v>
       </c>
       <c r="F46" t="n">
-        <v>155082428</v>
-      </c>
-      <c r="G46" t="n">
-        <v>38483582</v>
-      </c>
+        <v>5692767</v>
+      </c>
+      <c r="G46"/>
       <c r="H46" t="n">
-        <v>38770609</v>
+        <v>4193000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B47" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C47" t="n">
-        <v>74827</v>
-      </c>
-      <c r="D47" t="n">
-        <v>18557</v>
-      </c>
+        <v>1678</v>
+      </c>
+      <c r="D47"/>
       <c r="E47" t="n">
-        <v>18707</v>
+        <v>1062</v>
       </c>
       <c r="F47" t="n">
-        <v>213208583</v>
-      </c>
-      <c r="G47" t="n">
-        <v>54304484</v>
-      </c>
+        <v>5456082</v>
+      </c>
+      <c r="G47"/>
       <c r="H47" t="n">
-        <v>53302146</v>
+        <v>7278412</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B48" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C48" t="n">
-        <v>71394</v>
-      </c>
-      <c r="D48" t="n">
-        <v>17785</v>
-      </c>
+        <v>1411</v>
+      </c>
+      <c r="D48"/>
       <c r="E48" t="n">
-        <v>17849</v>
+        <v>1090</v>
       </c>
       <c r="F48" t="n">
-        <v>237492372</v>
-      </c>
-      <c r="G48" t="n">
-        <v>61035487</v>
-      </c>
+        <v>5590145</v>
+      </c>
+      <c r="G48"/>
       <c r="H48" t="n">
-        <v>59373100</v>
+        <v>4324052</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B49" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C49" t="n">
-        <v>77942</v>
+        <v>1882</v>
       </c>
       <c r="D49"/>
-      <c r="E49"/>
+      <c r="E49" t="n">
+        <v>849</v>
+      </c>
       <c r="F49" t="n">
-        <v>238497123</v>
+        <v>9178512</v>
       </c>
       <c r="G49"/>
-      <c r="H49"/>
+      <c r="H49" t="n">
+        <v>4323241</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B50" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C50" t="n">
-        <v>157536</v>
+        <v>1969</v>
       </c>
       <c r="D50"/>
       <c r="E50" t="n">
-        <v>39384</v>
+        <v>807</v>
       </c>
       <c r="F50" t="n">
-        <v>656865028</v>
+        <v>10627352</v>
       </c>
       <c r="G50"/>
       <c r="H50" t="n">
-        <v>164216257</v>
+        <v>4928630</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B51" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C51" t="n">
-        <v>159852</v>
+        <v>2104</v>
       </c>
       <c r="D51"/>
       <c r="E51" t="n">
-        <v>39963</v>
+        <v>921</v>
       </c>
       <c r="F51" t="n">
-        <v>636647852</v>
+        <v>11964815</v>
       </c>
       <c r="G51"/>
       <c r="H51" t="n">
-        <v>159161963</v>
+        <v>5737970</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B52" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="C52" t="n">
-        <v>131049</v>
+        <v>529500</v>
       </c>
       <c r="D52"/>
       <c r="E52" t="n">
-        <v>32762</v>
+        <v>132377</v>
       </c>
       <c r="F52" t="n">
-        <v>605719502</v>
+        <v>2144297005</v>
       </c>
       <c r="G52"/>
       <c r="H52" t="n">
-        <v>151429880</v>
+        <v>536073000</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B53" t="n">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="C53" t="n">
-        <v>143072</v>
+        <v>514992</v>
       </c>
       <c r="D53"/>
-      <c r="E53"/>
+      <c r="E53" t="n">
+        <v>128748</v>
+      </c>
       <c r="F53" t="n">
-        <v>812883432</v>
+        <v>2032237532</v>
       </c>
       <c r="G53"/>
-      <c r="H53"/>
+      <c r="H53" t="n">
+        <v>508057523</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B54" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C54" t="n">
-        <v>212544</v>
+        <v>523170</v>
       </c>
       <c r="D54"/>
-      <c r="E54"/>
+      <c r="E54" t="n">
+        <v>130793</v>
+      </c>
       <c r="F54" t="n">
-        <v>1461631935</v>
+        <v>2206987746</v>
       </c>
       <c r="G54"/>
-      <c r="H54"/>
+      <c r="H54" t="n">
+        <v>551758295</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B55" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C55" t="n">
-        <v>205392</v>
+        <v>574777</v>
       </c>
       <c r="D55"/>
-      <c r="E55"/>
+      <c r="E55" t="n">
+        <v>143694</v>
+      </c>
       <c r="F55" t="n">
-        <v>1570659426</v>
+        <v>2563437015</v>
       </c>
       <c r="G55"/>
-      <c r="H55"/>
+      <c r="H55" t="n">
+        <v>640859254</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B56" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C56" t="n">
-        <v>198408</v>
+        <v>561809</v>
       </c>
       <c r="D56"/>
-      <c r="E56"/>
+      <c r="E56" t="n">
+        <v>141333</v>
+      </c>
       <c r="F56" t="n">
-        <v>1866313911</v>
+        <v>3379295345</v>
       </c>
       <c r="G56"/>
-      <c r="H56"/>
+      <c r="H56" t="n">
+        <v>851690964</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B57" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C57" t="n">
-        <v>583549</v>
+        <v>563631</v>
       </c>
       <c r="D57"/>
       <c r="E57" t="n">
-        <v>145887</v>
+        <v>140908</v>
       </c>
       <c r="F57" t="n">
-        <v>2188954626</v>
+        <v>2735223696</v>
       </c>
       <c r="G57"/>
       <c r="H57" t="n">
-        <v>547238657</v>
+        <v>683805930</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B58" t="n">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="C58" t="n">
-        <v>521088</v>
+        <v>1274807</v>
       </c>
       <c r="D58"/>
       <c r="E58" t="n">
-        <v>130247</v>
+        <v>318596</v>
       </c>
       <c r="F58" t="n">
-        <v>2219984939</v>
+        <v>2599155441</v>
       </c>
       <c r="G58"/>
       <c r="H58" t="n">
-        <v>553121235</v>
+        <v>647819000</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B59" t="n">
-        <v>2023</v>
+        <v>2019</v>
       </c>
       <c r="C59" t="n">
-        <v>518985</v>
+        <v>1226030</v>
       </c>
       <c r="D59"/>
       <c r="E59" t="n">
-        <v>129746</v>
+        <v>306572</v>
       </c>
       <c r="F59" t="n">
-        <v>2473319380</v>
+        <v>2528870119</v>
       </c>
       <c r="G59"/>
       <c r="H59" t="n">
-        <v>618329840</v>
+        <v>633105946</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B60" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C60" t="n">
-        <v>19258</v>
+        <v>1089726</v>
       </c>
       <c r="D60"/>
       <c r="E60" t="n">
-        <v>4815</v>
+        <v>277185</v>
       </c>
       <c r="F60" t="n">
-        <v>60908930</v>
+        <v>2236212257</v>
       </c>
       <c r="G60"/>
       <c r="H60" t="n">
-        <v>15227232</v>
+        <v>581649799</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B61" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C61" t="n">
-        <v>17803</v>
+        <v>1106259</v>
       </c>
       <c r="D61"/>
       <c r="E61" t="n">
-        <v>4451</v>
+        <v>276565</v>
       </c>
       <c r="F61" t="n">
-        <v>74398339</v>
+        <v>2594433985</v>
       </c>
       <c r="G61"/>
       <c r="H61" t="n">
-        <v>18599583</v>
+        <v>648608496</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B62" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C62" t="n">
-        <v>14911</v>
+        <v>1090359</v>
       </c>
       <c r="D62"/>
       <c r="E62" t="n">
-        <v>3728</v>
+        <v>272990</v>
       </c>
       <c r="F62" t="n">
-        <v>66570692</v>
+        <v>3214508553</v>
       </c>
       <c r="G62"/>
       <c r="H62" t="n">
-        <v>16642670</v>
+        <v>808727377</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B63" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C63" t="n">
-        <v>16222</v>
+        <v>971014</v>
       </c>
       <c r="D63"/>
-      <c r="E63"/>
+      <c r="E63" t="n">
+        <v>242754</v>
+      </c>
       <c r="F63" t="n">
-        <v>65045692</v>
+        <v>3206663423</v>
       </c>
       <c r="G63"/>
-      <c r="H63"/>
+      <c r="H63" t="n">
+        <v>801665850</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B64" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C64" t="n">
-        <v>3608</v>
+        <v>57292</v>
       </c>
       <c r="D64"/>
       <c r="E64" t="n">
-        <v>902</v>
+        <v>14323</v>
       </c>
       <c r="F64" t="n">
-        <v>12657374</v>
+        <v>264325516</v>
       </c>
       <c r="G64"/>
       <c r="H64" t="n">
-        <v>3164343</v>
+        <v>66082000</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B65" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C65" t="n">
-        <v>3480</v>
+        <v>61183</v>
       </c>
       <c r="D65"/>
       <c r="E65" t="n">
-        <v>870</v>
+        <v>15296</v>
       </c>
       <c r="F65" t="n">
-        <v>13213450</v>
+        <v>249478738</v>
       </c>
       <c r="G65"/>
       <c r="H65" t="n">
-        <v>3303363</v>
+        <v>62369685</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B66" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C66" t="n">
-        <v>786</v>
+        <v>60212</v>
       </c>
       <c r="D66"/>
       <c r="E66" t="n">
-        <v>173</v>
+        <v>15053</v>
       </c>
       <c r="F66" t="n">
-        <v>3202921</v>
+        <v>232187250</v>
       </c>
       <c r="G66"/>
       <c r="H66" t="n">
-        <v>1038900</v>
+        <v>58046813</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B67" t="n">
         <v>2021</v>
       </c>
       <c r="C67" t="n">
-        <v>65641</v>
+        <v>57598</v>
       </c>
       <c r="D67"/>
       <c r="E67" t="n">
-        <v>16410</v>
+        <v>14399</v>
       </c>
       <c r="F67" t="n">
-        <v>840830294</v>
+        <v>262937076</v>
       </c>
       <c r="G67"/>
       <c r="H67" t="n">
-        <v>210207573</v>
+        <v>65734269</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B68" t="n">
         <v>2022</v>
       </c>
       <c r="C68" t="n">
-        <v>72202</v>
+        <v>65122</v>
       </c>
       <c r="D68"/>
       <c r="E68" t="n">
-        <v>18051</v>
+        <v>16280</v>
       </c>
       <c r="F68" t="n">
-        <v>1281736155</v>
+        <v>373857804</v>
       </c>
       <c r="G68"/>
       <c r="H68" t="n">
-        <v>320434039</v>
+        <v>93464451</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B69" t="n">
         <v>2023</v>
       </c>
       <c r="C69" t="n">
-        <v>83215</v>
+        <v>60674</v>
       </c>
       <c r="D69"/>
       <c r="E69" t="n">
-        <v>20804</v>
+        <v>15168</v>
       </c>
       <c r="F69" t="n">
-        <v>795793137</v>
+        <v>341522340</v>
       </c>
       <c r="G69"/>
       <c r="H69" t="n">
-        <v>198948280</v>
+        <v>85380590</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B70" t="n">
         <v>2024</v>
       </c>
       <c r="C70" t="n">
-        <v>76500</v>
+        <v>66465</v>
       </c>
       <c r="D70"/>
       <c r="E70"/>
       <c r="F70" t="n">
-        <v>767305344</v>
+        <v>346245538</v>
       </c>
       <c r="G70"/>
       <c r="H70"/>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B71" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C71" t="n">
-        <v>109754</v>
-      </c>
-      <c r="D71" t="n">
-        <v>40742</v>
-      </c>
+        <v>753310</v>
+      </c>
+      <c r="D71"/>
       <c r="E71" t="n">
-        <v>40527</v>
+        <v>188327</v>
       </c>
       <c r="F71" t="n">
-        <v>246230687</v>
-      </c>
-      <c r="G71" t="n">
-        <v>105762552</v>
-      </c>
+        <v>2755677252</v>
+      </c>
+      <c r="G71"/>
       <c r="H71" t="n">
-        <v>106793430</v>
+        <v>688914000</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B72" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C72" t="n">
-        <v>101701</v>
-      </c>
-      <c r="D72" t="n">
-        <v>38477</v>
-      </c>
+        <v>777313</v>
+      </c>
+      <c r="D72"/>
       <c r="E72" t="n">
-        <v>37894</v>
+        <v>194335</v>
       </c>
       <c r="F72" t="n">
-        <v>227145371</v>
-      </c>
-      <c r="G72" t="n">
-        <v>109912830</v>
-      </c>
+        <v>3034246123</v>
+      </c>
+      <c r="G72"/>
       <c r="H72" t="n">
-        <v>110689319</v>
+        <v>758655325</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B73" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C73" t="n">
-        <v>109417</v>
-      </c>
-      <c r="D73" t="n">
-        <v>41671</v>
-      </c>
+        <v>764207</v>
+      </c>
+      <c r="D73"/>
       <c r="E73" t="n">
-        <v>41221</v>
+        <v>191064</v>
       </c>
       <c r="F73" t="n">
-        <v>236842499</v>
-      </c>
-      <c r="G73" t="n">
-        <v>118679120</v>
-      </c>
+        <v>2889627722</v>
+      </c>
+      <c r="G73"/>
       <c r="H73" t="n">
-        <v>116711880</v>
+        <v>722586408</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B74" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C74" t="n">
-        <v>83824</v>
+        <v>773576</v>
       </c>
       <c r="D74"/>
-      <c r="E74"/>
+      <c r="E74" t="n">
+        <v>193394</v>
+      </c>
       <c r="F74" t="n">
-        <v>194350337</v>
+        <v>3124134782</v>
       </c>
       <c r="G74"/>
-      <c r="H74"/>
+      <c r="H74" t="n">
+        <v>781033695</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B75" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C75" t="n">
-        <v>6660448</v>
+        <v>736208</v>
       </c>
       <c r="D75"/>
-      <c r="E75"/>
+      <c r="E75" t="n">
+        <v>184052</v>
+      </c>
       <c r="F75" t="n">
-        <v>31659271257</v>
+        <v>3166130132</v>
       </c>
       <c r="G75"/>
-      <c r="H75"/>
+      <c r="H75" t="n">
+        <v>791532532</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B76" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C76" t="n">
-        <v>6646961</v>
+        <v>746246</v>
       </c>
       <c r="D76"/>
-      <c r="E76"/>
+      <c r="E76" t="n">
+        <v>186562</v>
+      </c>
       <c r="F76" t="n">
-        <v>42865428973</v>
+        <v>3622938207</v>
       </c>
       <c r="G76"/>
-      <c r="H76"/>
+      <c r="H76" t="n">
+        <v>905734580</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B77" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C77" t="n">
-        <v>6599860</v>
+        <v>725737</v>
       </c>
       <c r="D77"/>
       <c r="E77"/>
       <c r="F77" t="n">
-        <v>39997910616</v>
+        <v>3428948717</v>
       </c>
       <c r="G77"/>
       <c r="H77"/>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B78" t="n">
-        <v>2024</v>
+        <v>2018</v>
       </c>
       <c r="C78" t="n">
-        <v>3334500</v>
-      </c>
-      <c r="D78"/>
-      <c r="E78"/>
+        <v>78721</v>
+      </c>
+      <c r="D78" t="n">
+        <v>19680</v>
+      </c>
+      <c r="E78" t="n">
+        <v>19681</v>
+      </c>
       <c r="F78" t="n">
-        <v>19001323245</v>
-      </c>
-      <c r="G78"/>
-      <c r="H78"/>
+        <v>479915639</v>
+      </c>
+      <c r="G78" t="n">
+        <v>120484999</v>
+      </c>
+      <c r="H78" t="n">
+        <v>119981000</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B79" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C79" t="n">
-        <v>79220</v>
-      </c>
-      <c r="D79"/>
+        <v>81776</v>
+      </c>
+      <c r="D79" t="n">
+        <v>20443</v>
+      </c>
       <c r="E79" t="n">
-        <v>44787</v>
+        <v>20444</v>
       </c>
       <c r="F79" t="n">
-        <v>247203283</v>
-      </c>
-      <c r="G79"/>
+        <v>482748850</v>
+      </c>
+      <c r="G79" t="n">
+        <v>120773483</v>
+      </c>
       <c r="H79" t="n">
-        <v>159890251</v>
+        <v>120687212</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B80" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C80" t="n">
-        <v>84403</v>
-      </c>
-      <c r="D80"/>
+        <v>87083</v>
+      </c>
+      <c r="D80" t="n">
+        <v>21718</v>
+      </c>
       <c r="E80" t="n">
-        <v>42202</v>
+        <v>21771</v>
       </c>
       <c r="F80" t="n">
-        <v>371657647</v>
-      </c>
-      <c r="G80"/>
+        <v>531771831</v>
+      </c>
+      <c r="G80" t="n">
+        <v>133177094</v>
+      </c>
       <c r="H80" t="n">
-        <v>185828821</v>
+        <v>132947876</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B81" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C81" t="n">
-        <v>81333</v>
-      </c>
-      <c r="D81"/>
+        <v>123190</v>
+      </c>
+      <c r="D81" t="n">
+        <v>27920</v>
+      </c>
       <c r="E81" t="n">
-        <v>40667</v>
+        <v>26831</v>
       </c>
       <c r="F81" t="n">
-        <v>371776988</v>
-      </c>
-      <c r="G81"/>
+        <v>694026961</v>
+      </c>
+      <c r="G81" t="n">
+        <v>167033674</v>
+      </c>
       <c r="H81" t="n">
-        <v>185888510</v>
+        <v>162243534</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B82" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C82" t="n">
-        <v>70247</v>
-      </c>
-      <c r="D82"/>
+        <v>120127</v>
+      </c>
+      <c r="D82" t="n">
+        <v>27218</v>
+      </c>
       <c r="E82" t="n">
-        <v>17562</v>
+        <v>27197</v>
       </c>
       <c r="F82" t="n">
-        <v>631900238</v>
-      </c>
-      <c r="G82"/>
+        <v>740738278</v>
+      </c>
+      <c r="G82" t="n">
+        <v>177813277</v>
+      </c>
       <c r="H82" t="n">
-        <v>157975062</v>
+        <v>177097530</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B83" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C83" t="n">
-        <v>74753</v>
-      </c>
-      <c r="D83"/>
+        <v>84254</v>
+      </c>
+      <c r="D83" t="n">
+        <v>26824</v>
+      </c>
       <c r="E83" t="n">
-        <v>18683</v>
+        <v>26859</v>
       </c>
       <c r="F83" t="n">
-        <v>674132493</v>
-      </c>
-      <c r="G83"/>
+        <v>625028160</v>
+      </c>
+      <c r="G83" t="n">
+        <v>202702558</v>
+      </c>
       <c r="H83" t="n">
-        <v>168533125</v>
+        <v>203839780</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B84" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C84" t="n">
-        <v>73151</v>
+        <v>90884</v>
       </c>
       <c r="D84"/>
-      <c r="E84" t="n">
-        <v>18288</v>
-      </c>
+      <c r="E84"/>
       <c r="F84" t="n">
-        <v>846368614</v>
+        <v>595783690</v>
       </c>
       <c r="G84"/>
-      <c r="H84" t="n">
-        <v>211592200</v>
-      </c>
+      <c r="H84"/>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B85" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C85" t="n">
-        <v>46856</v>
+        <v>71602</v>
       </c>
       <c r="D85" t="n">
-        <v>11714</v>
+        <v>17852</v>
       </c>
       <c r="E85" t="n">
-        <v>11714</v>
+        <v>17899</v>
       </c>
       <c r="F85" t="n">
-        <v>143440009</v>
+        <v>155019979</v>
       </c>
       <c r="G85" t="n">
-        <v>36587679</v>
+        <v>38538333</v>
       </c>
       <c r="H85" t="n">
-        <v>35860002</v>
+        <v>38756000</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B86" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C86" t="n">
-        <v>44848</v>
+        <v>69260</v>
       </c>
       <c r="D86" t="n">
-        <v>11211</v>
+        <v>17283</v>
       </c>
       <c r="E86" t="n">
-        <v>11212</v>
+        <v>17315</v>
       </c>
       <c r="F86" t="n">
-        <v>164806847</v>
+        <v>143941353</v>
       </c>
       <c r="G86" t="n">
-        <v>36065959</v>
+        <v>35920179</v>
       </c>
       <c r="H86" t="n">
-        <v>41201711</v>
+        <v>35985337</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B87" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C87" t="n">
-        <v>45048</v>
+        <v>73540</v>
       </c>
       <c r="D87" t="n">
-        <v>11264</v>
+        <v>18436</v>
       </c>
       <c r="E87" t="n">
-        <v>11262</v>
+        <v>22210</v>
       </c>
       <c r="F87" t="n">
-        <v>191910568</v>
+        <v>139367550</v>
       </c>
       <c r="G87" t="n">
-        <v>37294481</v>
+        <v>35732770</v>
       </c>
       <c r="H87" t="n">
-        <v>47977660</v>
+        <v>41354066</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B88" t="n">
         <v>2021</v>
       </c>
       <c r="C88" t="n">
-        <v>60984</v>
-      </c>
-      <c r="D88"/>
+        <v>71823</v>
+      </c>
+      <c r="D88" t="n">
+        <v>18025</v>
+      </c>
       <c r="E88" t="n">
-        <v>15246</v>
+        <v>17956</v>
       </c>
       <c r="F88" t="n">
-        <v>59992594</v>
-      </c>
-      <c r="G88"/>
+        <v>155082428</v>
+      </c>
+      <c r="G88" t="n">
+        <v>38483582</v>
+      </c>
       <c r="H88" t="n">
-        <v>10616910</v>
+        <v>38770609</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B89" t="n">
         <v>2022</v>
       </c>
       <c r="C89" t="n">
-        <v>16492</v>
-      </c>
-      <c r="D89"/>
+        <v>74827</v>
+      </c>
+      <c r="D89" t="n">
+        <v>18557</v>
+      </c>
       <c r="E89" t="n">
-        <v>11327</v>
+        <v>18707</v>
       </c>
       <c r="F89" t="n">
-        <v>64700422</v>
-      </c>
-      <c r="G89"/>
+        <v>213208583</v>
+      </c>
+      <c r="G89" t="n">
+        <v>54304484</v>
+      </c>
       <c r="H89" t="n">
-        <v>57661416</v>
+        <v>53302146</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B90" t="n">
         <v>2023</v>
       </c>
       <c r="C90" t="n">
-        <v>15367</v>
-      </c>
-      <c r="D90"/>
+        <v>71394</v>
+      </c>
+      <c r="D90" t="n">
+        <v>17785</v>
+      </c>
       <c r="E90" t="n">
-        <v>11425</v>
+        <v>17849</v>
       </c>
       <c r="F90" t="n">
-        <v>57343590</v>
-      </c>
-      <c r="G90"/>
+        <v>237492372</v>
+      </c>
+      <c r="G90" t="n">
+        <v>61035487</v>
+      </c>
       <c r="H90" t="n">
-        <v>47532180</v>
+        <v>59373100</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B91" t="n">
         <v>2024</v>
       </c>
       <c r="C91" t="n">
-        <v>28929</v>
+        <v>77942</v>
       </c>
       <c r="D91"/>
       <c r="E91"/>
       <c r="F91" t="n">
-        <v>134867441</v>
+        <v>238497123</v>
       </c>
       <c r="G91"/>
       <c r="H91"/>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B92" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C92" t="n">
-        <v>6768</v>
+        <v>139067</v>
       </c>
       <c r="D92"/>
       <c r="E92" t="n">
-        <v>1692</v>
+        <v>34605</v>
       </c>
       <c r="F92" t="n">
-        <v>24508684</v>
+        <v>661716886</v>
       </c>
       <c r="G92"/>
       <c r="H92" t="n">
-        <v>6127171</v>
+        <v>164936000</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B93" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C93" t="n">
-        <v>4593</v>
+        <v>139908</v>
       </c>
       <c r="D93"/>
       <c r="E93" t="n">
-        <v>1644</v>
+        <v>34977</v>
       </c>
       <c r="F93" t="n">
-        <v>13161018</v>
+        <v>630653564</v>
       </c>
       <c r="G93"/>
       <c r="H93" t="n">
-        <v>6861528</v>
+        <v>157663391</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B94" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C94" t="n">
-        <v>2681</v>
+        <v>140608</v>
       </c>
       <c r="D94"/>
       <c r="E94" t="n">
-        <v>1108</v>
+        <v>35183</v>
       </c>
       <c r="F94" t="n">
-        <v>13337722</v>
+        <v>649751524</v>
       </c>
       <c r="G94"/>
       <c r="H94" t="n">
-        <v>5346310</v>
+        <v>162667517</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B95" t="n">
         <v>2021</v>
       </c>
       <c r="C95" t="n">
-        <v>9670</v>
+        <v>157536</v>
       </c>
       <c r="D95"/>
       <c r="E95" t="n">
-        <v>2352</v>
+        <v>39384</v>
       </c>
       <c r="F95" t="n">
-        <v>27963598</v>
+        <v>656865028</v>
       </c>
       <c r="G95"/>
       <c r="H95" t="n">
-        <v>6725843</v>
+        <v>164216257</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B96" t="n">
         <v>2022</v>
       </c>
       <c r="C96" t="n">
-        <v>10723</v>
+        <v>159852</v>
       </c>
       <c r="D96"/>
       <c r="E96" t="n">
-        <v>2681</v>
+        <v>39963</v>
       </c>
       <c r="F96" t="n">
-        <v>32245006</v>
+        <v>636647852</v>
       </c>
       <c r="G96"/>
       <c r="H96" t="n">
-        <v>8061252</v>
+        <v>159161963</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B97" t="n">
         <v>2023</v>
       </c>
       <c r="C97" t="n">
-        <v>11073</v>
+        <v>131049</v>
       </c>
       <c r="D97"/>
       <c r="E97" t="n">
-        <v>2768</v>
+        <v>32762</v>
       </c>
       <c r="F97" t="n">
-        <v>35816654</v>
+        <v>605719502</v>
       </c>
       <c r="G97"/>
       <c r="H97" t="n">
-        <v>8954160</v>
+        <v>151429880</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B98" t="n">
         <v>2024</v>
       </c>
       <c r="C98" t="n">
-        <v>10275</v>
+        <v>143072</v>
       </c>
       <c r="D98"/>
       <c r="E98"/>
       <c r="F98" t="n">
-        <v>36596063</v>
+        <v>812883432</v>
       </c>
       <c r="G98"/>
       <c r="H98"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="s">
+        <v>23</v>
+      </c>
+      <c r="B99" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C99" t="n">
+        <v>75176</v>
+      </c>
+      <c r="D99"/>
+      <c r="E99"/>
+      <c r="F99" t="n">
+        <v>62357023</v>
+      </c>
+      <c r="G99"/>
+      <c r="H99"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="s">
+        <v>23</v>
+      </c>
+      <c r="B100" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C100" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100"/>
+      <c r="E100"/>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100"/>
+      <c r="H100"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="s">
+        <v>23</v>
+      </c>
+      <c r="B101" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C101" t="n">
+        <v>205392</v>
+      </c>
+      <c r="D101"/>
+      <c r="E101"/>
+      <c r="F101" t="n">
+        <v>1445181420</v>
+      </c>
+      <c r="G101"/>
+      <c r="H101"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="s">
+        <v>23</v>
+      </c>
+      <c r="B102" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C102" t="n">
+        <v>212544</v>
+      </c>
+      <c r="D102"/>
+      <c r="E102"/>
+      <c r="F102" t="n">
+        <v>1461631935</v>
+      </c>
+      <c r="G102"/>
+      <c r="H102"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="s">
+        <v>23</v>
+      </c>
+      <c r="B103" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C103" t="n">
+        <v>205392</v>
+      </c>
+      <c r="D103"/>
+      <c r="E103"/>
+      <c r="F103" t="n">
+        <v>1570659426</v>
+      </c>
+      <c r="G103"/>
+      <c r="H103"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="s">
+        <v>23</v>
+      </c>
+      <c r="B104" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C104" t="n">
+        <v>198408</v>
+      </c>
+      <c r="D104"/>
+      <c r="E104"/>
+      <c r="F104" t="n">
+        <v>1866313911</v>
+      </c>
+      <c r="G104"/>
+      <c r="H104"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="s">
+        <v>24</v>
+      </c>
+      <c r="B105" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C105" t="n">
+        <v>570906</v>
+      </c>
+      <c r="D105"/>
+      <c r="E105" t="n">
+        <v>142727</v>
+      </c>
+      <c r="F105" t="n">
+        <v>1756558633</v>
+      </c>
+      <c r="G105"/>
+      <c r="H105" t="n">
+        <v>439139000</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s">
+        <v>24</v>
+      </c>
+      <c r="B106" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C106" t="n">
+        <v>529111</v>
+      </c>
+      <c r="D106"/>
+      <c r="E106" t="n">
+        <v>132278</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1783430447</v>
+      </c>
+      <c r="G106"/>
+      <c r="H106" t="n">
+        <v>445857612</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s">
+        <v>24</v>
+      </c>
+      <c r="B107" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C107" t="n">
+        <v>490969</v>
+      </c>
+      <c r="D107"/>
+      <c r="E107" t="n">
+        <v>122744</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1566633128</v>
+      </c>
+      <c r="G107"/>
+      <c r="H107" t="n">
+        <v>391700279</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
+        <v>24</v>
+      </c>
+      <c r="B108" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C108" t="n">
+        <v>583549</v>
+      </c>
+      <c r="D108"/>
+      <c r="E108" t="n">
+        <v>145887</v>
+      </c>
+      <c r="F108" t="n">
+        <v>2188954626</v>
+      </c>
+      <c r="G108"/>
+      <c r="H108" t="n">
+        <v>547238657</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s">
+        <v>24</v>
+      </c>
+      <c r="B109" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C109" t="n">
+        <v>521088</v>
+      </c>
+      <c r="D109"/>
+      <c r="E109" t="n">
+        <v>130247</v>
+      </c>
+      <c r="F109" t="n">
+        <v>2219984939</v>
+      </c>
+      <c r="G109"/>
+      <c r="H109" t="n">
+        <v>553121235</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
+        <v>24</v>
+      </c>
+      <c r="B110" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C110" t="n">
+        <v>518985</v>
+      </c>
+      <c r="D110"/>
+      <c r="E110" t="n">
+        <v>129746</v>
+      </c>
+      <c r="F110" t="n">
+        <v>2473319380</v>
+      </c>
+      <c r="G110"/>
+      <c r="H110" t="n">
+        <v>618329840</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s">
+        <v>25</v>
+      </c>
+      <c r="B111" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C111" t="n">
+        <v>13800</v>
+      </c>
+      <c r="D111"/>
+      <c r="E111" t="n">
+        <v>3450</v>
+      </c>
+      <c r="F111" t="n">
+        <v>44947398</v>
+      </c>
+      <c r="G111"/>
+      <c r="H111" t="n">
+        <v>11238000</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>25</v>
+      </c>
+      <c r="B112" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C112" t="n">
+        <v>15101</v>
+      </c>
+      <c r="D112"/>
+      <c r="E112" t="n">
+        <v>3776</v>
+      </c>
+      <c r="F112" t="n">
+        <v>47900885</v>
+      </c>
+      <c r="G112"/>
+      <c r="H112" t="n">
+        <v>11982026</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s">
+        <v>25</v>
+      </c>
+      <c r="B113" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C113" t="n">
+        <v>16278</v>
+      </c>
+      <c r="D113"/>
+      <c r="E113" t="n">
+        <v>3975</v>
+      </c>
+      <c r="F113" t="n">
+        <v>50021879</v>
+      </c>
+      <c r="G113"/>
+      <c r="H113" t="n">
+        <v>12042994</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
+        <v>25</v>
+      </c>
+      <c r="B114" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C114" t="n">
+        <v>19258</v>
+      </c>
+      <c r="D114"/>
+      <c r="E114" t="n">
+        <v>4815</v>
+      </c>
+      <c r="F114" t="n">
+        <v>60908930</v>
+      </c>
+      <c r="G114"/>
+      <c r="H114" t="n">
+        <v>15227232</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s">
+        <v>25</v>
+      </c>
+      <c r="B115" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C115" t="n">
+        <v>17803</v>
+      </c>
+      <c r="D115"/>
+      <c r="E115" t="n">
+        <v>4451</v>
+      </c>
+      <c r="F115" t="n">
+        <v>74398339</v>
+      </c>
+      <c r="G115"/>
+      <c r="H115" t="n">
+        <v>18599583</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
+        <v>25</v>
+      </c>
+      <c r="B116" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C116" t="n">
+        <v>14911</v>
+      </c>
+      <c r="D116"/>
+      <c r="E116" t="n">
+        <v>3728</v>
+      </c>
+      <c r="F116" t="n">
+        <v>66570692</v>
+      </c>
+      <c r="G116"/>
+      <c r="H116" t="n">
+        <v>16642670</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s">
+        <v>25</v>
+      </c>
+      <c r="B117" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C117" t="n">
+        <v>16222</v>
+      </c>
+      <c r="D117"/>
+      <c r="E117"/>
+      <c r="F117" t="n">
+        <v>65045692</v>
+      </c>
+      <c r="G117"/>
+      <c r="H117"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="s">
+        <v>26</v>
+      </c>
+      <c r="B118" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C118" t="n">
+        <v>2168</v>
+      </c>
+      <c r="D118"/>
+      <c r="E118" t="n">
+        <v>962</v>
+      </c>
+      <c r="F118" t="n">
+        <v>5102494</v>
+      </c>
+      <c r="G118"/>
+      <c r="H118" t="n">
+        <v>2194000</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s">
+        <v>26</v>
+      </c>
+      <c r="B119" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C119" t="n">
+        <v>2505</v>
+      </c>
+      <c r="D119"/>
+      <c r="E119" t="n">
+        <v>628</v>
+      </c>
+      <c r="F119" t="n">
+        <v>7388248</v>
+      </c>
+      <c r="G119"/>
+      <c r="H119" t="n">
+        <v>1852373</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
+        <v>26</v>
+      </c>
+      <c r="B120" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C120" t="n">
+        <v>2910</v>
+      </c>
+      <c r="D120"/>
+      <c r="E120" t="n">
+        <v>727</v>
+      </c>
+      <c r="F120" t="n">
+        <v>9007310</v>
+      </c>
+      <c r="G120"/>
+      <c r="H120" t="n">
+        <v>2251828</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s">
+        <v>26</v>
+      </c>
+      <c r="B121" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C121" t="n">
+        <v>3608</v>
+      </c>
+      <c r="D121"/>
+      <c r="E121" t="n">
+        <v>902</v>
+      </c>
+      <c r="F121" t="n">
+        <v>12657374</v>
+      </c>
+      <c r="G121"/>
+      <c r="H121" t="n">
+        <v>3164343</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>26</v>
+      </c>
+      <c r="B122" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C122" t="n">
+        <v>3480</v>
+      </c>
+      <c r="D122"/>
+      <c r="E122" t="n">
+        <v>870</v>
+      </c>
+      <c r="F122" t="n">
+        <v>13213450</v>
+      </c>
+      <c r="G122"/>
+      <c r="H122" t="n">
+        <v>3303363</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>26</v>
+      </c>
+      <c r="B123" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C123" t="n">
+        <v>786</v>
+      </c>
+      <c r="D123"/>
+      <c r="E123" t="n">
+        <v>173</v>
+      </c>
+      <c r="F123" t="n">
+        <v>3202921</v>
+      </c>
+      <c r="G123"/>
+      <c r="H123" t="n">
+        <v>1038900</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>27</v>
+      </c>
+      <c r="B124" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C124" t="n">
+        <v>77166</v>
+      </c>
+      <c r="D124"/>
+      <c r="E124" t="n">
+        <v>19292</v>
+      </c>
+      <c r="F124" t="n">
+        <v>970737803</v>
+      </c>
+      <c r="G124"/>
+      <c r="H124" t="n">
+        <v>242683000</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>27</v>
+      </c>
+      <c r="B125" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C125" t="n">
+        <v>55294</v>
+      </c>
+      <c r="D125"/>
+      <c r="E125" t="n">
+        <v>13823</v>
+      </c>
+      <c r="F125" t="n">
+        <v>647648820</v>
+      </c>
+      <c r="G125"/>
+      <c r="H125" t="n">
+        <v>161912205</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>27</v>
+      </c>
+      <c r="B126" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C126" t="n">
+        <v>79318</v>
+      </c>
+      <c r="D126"/>
+      <c r="E126" t="n">
+        <v>19829</v>
+      </c>
+      <c r="F126" t="n">
+        <v>861787061</v>
+      </c>
+      <c r="G126"/>
+      <c r="H126" t="n">
+        <v>215446765</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>27</v>
+      </c>
+      <c r="B127" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C127" t="n">
+        <v>65641</v>
+      </c>
+      <c r="D127"/>
+      <c r="E127" t="n">
+        <v>16410</v>
+      </c>
+      <c r="F127" t="n">
+        <v>840830294</v>
+      </c>
+      <c r="G127"/>
+      <c r="H127" t="n">
+        <v>210207573</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>27</v>
+      </c>
+      <c r="B128" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C128" t="n">
+        <v>72202</v>
+      </c>
+      <c r="D128"/>
+      <c r="E128" t="n">
+        <v>18051</v>
+      </c>
+      <c r="F128" t="n">
+        <v>1281736155</v>
+      </c>
+      <c r="G128"/>
+      <c r="H128" t="n">
+        <v>320434039</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>27</v>
+      </c>
+      <c r="B129" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C129" t="n">
+        <v>83215</v>
+      </c>
+      <c r="D129"/>
+      <c r="E129" t="n">
+        <v>20804</v>
+      </c>
+      <c r="F129" t="n">
+        <v>795793137</v>
+      </c>
+      <c r="G129"/>
+      <c r="H129" t="n">
+        <v>198948280</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s">
+        <v>27</v>
+      </c>
+      <c r="B130" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C130" t="n">
+        <v>76500</v>
+      </c>
+      <c r="D130"/>
+      <c r="E130"/>
+      <c r="F130" t="n">
+        <v>767305344</v>
+      </c>
+      <c r="G130"/>
+      <c r="H130"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="s">
+        <v>28</v>
+      </c>
+      <c r="B131" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C131" t="n">
+        <v>212016</v>
+      </c>
+      <c r="D131" t="n">
+        <v>53542</v>
+      </c>
+      <c r="E131" t="n">
+        <v>53004</v>
+      </c>
+      <c r="F131" t="n">
+        <v>382203366</v>
+      </c>
+      <c r="G131" t="n">
+        <v>99954716</v>
+      </c>
+      <c r="H131" t="n">
+        <v>95551000</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s">
+        <v>28</v>
+      </c>
+      <c r="B132" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C132" t="n">
+        <v>125441</v>
+      </c>
+      <c r="D132" t="n">
+        <v>45987</v>
+      </c>
+      <c r="E132" t="n">
+        <v>46340</v>
+      </c>
+      <c r="F132" t="n">
+        <v>185043131</v>
+      </c>
+      <c r="G132" t="n">
+        <v>95547671</v>
+      </c>
+      <c r="H132" t="n">
+        <v>84052015</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="s">
+        <v>28</v>
+      </c>
+      <c r="B133" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C133" t="n">
+        <v>108143</v>
+      </c>
+      <c r="D133" t="n">
+        <v>40052</v>
+      </c>
+      <c r="E133" t="n">
+        <v>40168</v>
+      </c>
+      <c r="F133" t="n">
+        <v>187781439</v>
+      </c>
+      <c r="G133" t="n">
+        <v>92833441</v>
+      </c>
+      <c r="H133" t="n">
+        <v>85509274</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="s">
+        <v>28</v>
+      </c>
+      <c r="B134" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C134" t="n">
+        <v>109754</v>
+      </c>
+      <c r="D134" t="n">
+        <v>40742</v>
+      </c>
+      <c r="E134" t="n">
+        <v>40527</v>
+      </c>
+      <c r="F134" t="n">
+        <v>246230687</v>
+      </c>
+      <c r="G134" t="n">
+        <v>105762552</v>
+      </c>
+      <c r="H134" t="n">
+        <v>106793430</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="s">
+        <v>28</v>
+      </c>
+      <c r="B135" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C135" t="n">
+        <v>101701</v>
+      </c>
+      <c r="D135" t="n">
+        <v>38477</v>
+      </c>
+      <c r="E135" t="n">
+        <v>37894</v>
+      </c>
+      <c r="F135" t="n">
+        <v>227145371</v>
+      </c>
+      <c r="G135" t="n">
+        <v>109912830</v>
+      </c>
+      <c r="H135" t="n">
+        <v>110689319</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s">
+        <v>28</v>
+      </c>
+      <c r="B136" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C136" t="n">
+        <v>109417</v>
+      </c>
+      <c r="D136" t="n">
+        <v>41671</v>
+      </c>
+      <c r="E136" t="n">
+        <v>41221</v>
+      </c>
+      <c r="F136" t="n">
+        <v>236842499</v>
+      </c>
+      <c r="G136" t="n">
+        <v>118679120</v>
+      </c>
+      <c r="H136" t="n">
+        <v>116711880</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="s">
+        <v>28</v>
+      </c>
+      <c r="B137" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C137" t="n">
+        <v>83824</v>
+      </c>
+      <c r="D137"/>
+      <c r="E137"/>
+      <c r="F137" t="n">
+        <v>194350337</v>
+      </c>
+      <c r="G137"/>
+      <c r="H137"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="s">
+        <v>29</v>
+      </c>
+      <c r="B138" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C138" t="n">
+        <v>5420460</v>
+      </c>
+      <c r="D138"/>
+      <c r="E138"/>
+      <c r="F138" t="n">
+        <v>28275781732</v>
+      </c>
+      <c r="G138"/>
+      <c r="H138"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="s">
+        <v>29</v>
+      </c>
+      <c r="B139" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C139" t="n">
+        <v>5812170</v>
+      </c>
+      <c r="D139"/>
+      <c r="E139"/>
+      <c r="F139" t="n">
+        <v>29128321005</v>
+      </c>
+      <c r="G139"/>
+      <c r="H139"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="s">
+        <v>29</v>
+      </c>
+      <c r="B140" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C140" t="n">
+        <v>5961648</v>
+      </c>
+      <c r="D140"/>
+      <c r="E140"/>
+      <c r="F140" t="n">
+        <v>25642854707</v>
+      </c>
+      <c r="G140"/>
+      <c r="H140"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="s">
+        <v>29</v>
+      </c>
+      <c r="B141" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C141" t="n">
+        <v>6660448</v>
+      </c>
+      <c r="D141"/>
+      <c r="E141"/>
+      <c r="F141" t="n">
+        <v>31659271257</v>
+      </c>
+      <c r="G141"/>
+      <c r="H141"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="s">
+        <v>29</v>
+      </c>
+      <c r="B142" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C142" t="n">
+        <v>6646961</v>
+      </c>
+      <c r="D142"/>
+      <c r="E142"/>
+      <c r="F142" t="n">
+        <v>42865428973</v>
+      </c>
+      <c r="G142"/>
+      <c r="H142"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="s">
+        <v>29</v>
+      </c>
+      <c r="B143" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C143" t="n">
+        <v>6599860</v>
+      </c>
+      <c r="D143"/>
+      <c r="E143"/>
+      <c r="F143" t="n">
+        <v>39997910616</v>
+      </c>
+      <c r="G143"/>
+      <c r="H143"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="s">
+        <v>29</v>
+      </c>
+      <c r="B144" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C144" t="n">
+        <v>3334500</v>
+      </c>
+      <c r="D144"/>
+      <c r="E144"/>
+      <c r="F144" t="n">
+        <v>19001323245</v>
+      </c>
+      <c r="G144"/>
+      <c r="H144"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="s">
+        <v>30</v>
+      </c>
+      <c r="B145" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C145" t="n">
+        <v>147225</v>
+      </c>
+      <c r="D145"/>
+      <c r="E145" t="n">
+        <v>36804</v>
+      </c>
+      <c r="F145" t="n">
+        <v>418668404</v>
+      </c>
+      <c r="G145"/>
+      <c r="H145" t="n">
+        <v>104668000</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="s">
+        <v>30</v>
+      </c>
+      <c r="B146" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C146" t="n">
+        <v>158922</v>
+      </c>
+      <c r="D146"/>
+      <c r="E146" t="n">
+        <v>42627</v>
+      </c>
+      <c r="F146" t="n">
+        <v>416765491</v>
+      </c>
+      <c r="G146"/>
+      <c r="H146" t="n">
+        <v>114755930</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="s">
+        <v>30</v>
+      </c>
+      <c r="B147" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C147" t="n">
+        <v>181671</v>
+      </c>
+      <c r="D147"/>
+      <c r="E147" t="n">
+        <v>45968</v>
+      </c>
+      <c r="F147" t="n">
+        <v>484137649</v>
+      </c>
+      <c r="G147"/>
+      <c r="H147" t="n">
+        <v>122684403</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="s">
+        <v>30</v>
+      </c>
+      <c r="B148" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C148" t="n">
+        <v>79220</v>
+      </c>
+      <c r="D148"/>
+      <c r="E148" t="n">
+        <v>44787</v>
+      </c>
+      <c r="F148" t="n">
+        <v>247203283</v>
+      </c>
+      <c r="G148"/>
+      <c r="H148" t="n">
+        <v>159890251</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="s">
+        <v>30</v>
+      </c>
+      <c r="B149" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C149" t="n">
+        <v>84403</v>
+      </c>
+      <c r="D149"/>
+      <c r="E149" t="n">
+        <v>42202</v>
+      </c>
+      <c r="F149" t="n">
+        <v>371657647</v>
+      </c>
+      <c r="G149"/>
+      <c r="H149" t="n">
+        <v>185828821</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="s">
+        <v>30</v>
+      </c>
+      <c r="B150" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C150" t="n">
+        <v>81333</v>
+      </c>
+      <c r="D150"/>
+      <c r="E150" t="n">
+        <v>40667</v>
+      </c>
+      <c r="F150" t="n">
+        <v>371776988</v>
+      </c>
+      <c r="G150"/>
+      <c r="H150" t="n">
+        <v>185888510</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="s">
+        <v>31</v>
+      </c>
+      <c r="B151" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C151" t="n">
+        <v>47064</v>
+      </c>
+      <c r="D151"/>
+      <c r="E151" t="n">
+        <v>13512</v>
+      </c>
+      <c r="F151" t="n">
+        <v>387292488</v>
+      </c>
+      <c r="G151"/>
+      <c r="H151" t="n">
+        <v>98570000</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="s">
+        <v>31</v>
+      </c>
+      <c r="B152" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C152" t="n">
+        <v>51523</v>
+      </c>
+      <c r="D152"/>
+      <c r="E152" t="n">
+        <v>12881</v>
+      </c>
+      <c r="F152" t="n">
+        <v>432118594</v>
+      </c>
+      <c r="G152"/>
+      <c r="H152" t="n">
+        <v>108029649</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="s">
+        <v>31</v>
+      </c>
+      <c r="B153" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C153" t="n">
+        <v>54591</v>
+      </c>
+      <c r="D153"/>
+      <c r="E153" t="n">
+        <v>17206</v>
+      </c>
+      <c r="F153" t="n">
+        <v>390127295</v>
+      </c>
+      <c r="G153"/>
+      <c r="H153" t="n">
+        <v>121441034</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="s">
+        <v>31</v>
+      </c>
+      <c r="B154" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C154" t="n">
+        <v>70247</v>
+      </c>
+      <c r="D154"/>
+      <c r="E154" t="n">
+        <v>17562</v>
+      </c>
+      <c r="F154" t="n">
+        <v>631900238</v>
+      </c>
+      <c r="G154"/>
+      <c r="H154" t="n">
+        <v>157975062</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="s">
+        <v>31</v>
+      </c>
+      <c r="B155" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C155" t="n">
+        <v>74753</v>
+      </c>
+      <c r="D155"/>
+      <c r="E155" t="n">
+        <v>18683</v>
+      </c>
+      <c r="F155" t="n">
+        <v>674132493</v>
+      </c>
+      <c r="G155"/>
+      <c r="H155" t="n">
+        <v>168533125</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="s">
+        <v>31</v>
+      </c>
+      <c r="B156" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C156" t="n">
+        <v>73151</v>
+      </c>
+      <c r="D156"/>
+      <c r="E156" t="n">
+        <v>18288</v>
+      </c>
+      <c r="F156" t="n">
+        <v>846368614</v>
+      </c>
+      <c r="G156"/>
+      <c r="H156" t="n">
+        <v>211592200</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="s">
+        <v>32</v>
+      </c>
+      <c r="B157" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C157" t="n">
+        <v>49194</v>
+      </c>
+      <c r="D157" t="n">
+        <v>12298</v>
+      </c>
+      <c r="E157" t="n">
+        <v>12300</v>
+      </c>
+      <c r="F157" t="n">
+        <v>134230778</v>
+      </c>
+      <c r="G157" t="n">
+        <v>30720828</v>
+      </c>
+      <c r="H157" t="n">
+        <v>33559000</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="s">
+        <v>32</v>
+      </c>
+      <c r="B158" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C158" t="n">
+        <v>50512</v>
+      </c>
+      <c r="D158" t="n">
+        <v>12848</v>
+      </c>
+      <c r="E158" t="n">
+        <v>12628</v>
+      </c>
+      <c r="F158" t="n">
+        <v>149937833</v>
+      </c>
+      <c r="G158" t="n">
+        <v>31754832</v>
+      </c>
+      <c r="H158" t="n">
+        <v>37484459</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="s">
+        <v>32</v>
+      </c>
+      <c r="B159" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C159" t="n">
+        <v>48600</v>
+      </c>
+      <c r="D159" t="n">
+        <v>12371</v>
+      </c>
+      <c r="E159" t="n">
+        <v>12078</v>
+      </c>
+      <c r="F159" t="n">
+        <v>155951471</v>
+      </c>
+      <c r="G159" t="n">
+        <v>39470089</v>
+      </c>
+      <c r="H159" t="n">
+        <v>38789821</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="s">
+        <v>32</v>
+      </c>
+      <c r="B160" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C160" t="n">
+        <v>46856</v>
+      </c>
+      <c r="D160" t="n">
+        <v>11714</v>
+      </c>
+      <c r="E160" t="n">
+        <v>11714</v>
+      </c>
+      <c r="F160" t="n">
+        <v>143440009</v>
+      </c>
+      <c r="G160" t="n">
+        <v>36587679</v>
+      </c>
+      <c r="H160" t="n">
+        <v>35860002</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="s">
+        <v>32</v>
+      </c>
+      <c r="B161" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C161" t="n">
+        <v>44848</v>
+      </c>
+      <c r="D161" t="n">
+        <v>11211</v>
+      </c>
+      <c r="E161" t="n">
+        <v>11212</v>
+      </c>
+      <c r="F161" t="n">
+        <v>164806847</v>
+      </c>
+      <c r="G161" t="n">
+        <v>36065959</v>
+      </c>
+      <c r="H161" t="n">
+        <v>41201711</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="s">
+        <v>32</v>
+      </c>
+      <c r="B162" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C162" t="n">
+        <v>45048</v>
+      </c>
+      <c r="D162" t="n">
+        <v>11264</v>
+      </c>
+      <c r="E162" t="n">
+        <v>11262</v>
+      </c>
+      <c r="F162" t="n">
+        <v>191910568</v>
+      </c>
+      <c r="G162" t="n">
+        <v>37294481</v>
+      </c>
+      <c r="H162" t="n">
+        <v>47977660</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="s">
+        <v>33</v>
+      </c>
+      <c r="B163" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C163" t="n">
+        <v>33013</v>
+      </c>
+      <c r="D163"/>
+      <c r="E163" t="n">
+        <v>11671</v>
+      </c>
+      <c r="F163" t="n">
+        <v>119186103</v>
+      </c>
+      <c r="G163"/>
+      <c r="H163" t="n">
+        <v>41212000</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s">
+        <v>33</v>
+      </c>
+      <c r="B164" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C164" t="n">
+        <v>25369</v>
+      </c>
+      <c r="D164"/>
+      <c r="E164" t="n">
+        <v>11497</v>
+      </c>
+      <c r="F164" t="n">
+        <v>82626287</v>
+      </c>
+      <c r="G164"/>
+      <c r="H164" t="n">
+        <v>34827448</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="s">
+        <v>33</v>
+      </c>
+      <c r="B165" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C165" t="n">
+        <v>48357</v>
+      </c>
+      <c r="D165"/>
+      <c r="E165" t="n">
+        <v>12089</v>
+      </c>
+      <c r="F165" t="n">
+        <v>139755106</v>
+      </c>
+      <c r="G165"/>
+      <c r="H165" t="n">
+        <v>34938768</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="s">
+        <v>33</v>
+      </c>
+      <c r="B166" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C166" t="n">
+        <v>60984</v>
+      </c>
+      <c r="D166"/>
+      <c r="E166" t="n">
+        <v>15246</v>
+      </c>
+      <c r="F166" t="n">
+        <v>59992594</v>
+      </c>
+      <c r="G166"/>
+      <c r="H166" t="n">
+        <v>10616910</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="s">
+        <v>33</v>
+      </c>
+      <c r="B167" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C167" t="n">
+        <v>16492</v>
+      </c>
+      <c r="D167"/>
+      <c r="E167" t="n">
+        <v>11327</v>
+      </c>
+      <c r="F167" t="n">
+        <v>64700422</v>
+      </c>
+      <c r="G167"/>
+      <c r="H167" t="n">
+        <v>57661416</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="s">
+        <v>33</v>
+      </c>
+      <c r="B168" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C168" t="n">
+        <v>15367</v>
+      </c>
+      <c r="D168"/>
+      <c r="E168" t="n">
+        <v>11425</v>
+      </c>
+      <c r="F168" t="n">
+        <v>57343590</v>
+      </c>
+      <c r="G168"/>
+      <c r="H168" t="n">
+        <v>47532180</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="s">
+        <v>33</v>
+      </c>
+      <c r="B169" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C169" t="n">
+        <v>28929</v>
+      </c>
+      <c r="D169"/>
+      <c r="E169"/>
+      <c r="F169" t="n">
+        <v>134867441</v>
+      </c>
+      <c r="G169"/>
+      <c r="H169"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="s">
+        <v>34</v>
+      </c>
+      <c r="B170" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C170" t="n">
+        <v>3096</v>
+      </c>
+      <c r="D170"/>
+      <c r="E170" t="n">
+        <v>1763</v>
+      </c>
+      <c r="F170" t="n">
+        <v>6971056</v>
+      </c>
+      <c r="G170"/>
+      <c r="H170" t="n">
+        <v>5467000</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="s">
+        <v>34</v>
+      </c>
+      <c r="B171" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C171" t="n">
+        <v>3807</v>
+      </c>
+      <c r="D171"/>
+      <c r="E171" t="n">
+        <v>2087</v>
+      </c>
+      <c r="F171" t="n">
+        <v>8355821</v>
+      </c>
+      <c r="G171"/>
+      <c r="H171" t="n">
+        <v>6092754</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="s">
+        <v>34</v>
+      </c>
+      <c r="B172" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C172" t="n">
+        <v>6696</v>
+      </c>
+      <c r="D172"/>
+      <c r="E172" t="n">
+        <v>1936</v>
+      </c>
+      <c r="F172" t="n">
+        <v>6752817</v>
+      </c>
+      <c r="G172"/>
+      <c r="H172" t="n">
+        <v>5674246</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="s">
+        <v>34</v>
+      </c>
+      <c r="B173" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C173" t="n">
+        <v>6768</v>
+      </c>
+      <c r="D173"/>
+      <c r="E173" t="n">
+        <v>1692</v>
+      </c>
+      <c r="F173" t="n">
+        <v>24508684</v>
+      </c>
+      <c r="G173"/>
+      <c r="H173" t="n">
+        <v>6127171</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="s">
+        <v>34</v>
+      </c>
+      <c r="B174" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C174" t="n">
+        <v>4593</v>
+      </c>
+      <c r="D174"/>
+      <c r="E174" t="n">
+        <v>1644</v>
+      </c>
+      <c r="F174" t="n">
+        <v>13161018</v>
+      </c>
+      <c r="G174"/>
+      <c r="H174" t="n">
+        <v>6861528</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="s">
+        <v>34</v>
+      </c>
+      <c r="B175" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C175" t="n">
+        <v>2681</v>
+      </c>
+      <c r="D175"/>
+      <c r="E175" t="n">
+        <v>1108</v>
+      </c>
+      <c r="F175" t="n">
+        <v>13337722</v>
+      </c>
+      <c r="G175"/>
+      <c r="H175" t="n">
+        <v>5346310</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="s">
+        <v>35</v>
+      </c>
+      <c r="B176" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C176" t="n">
+        <v>8988</v>
+      </c>
+      <c r="D176"/>
+      <c r="E176" t="n">
+        <v>2247</v>
+      </c>
+      <c r="F176" t="n">
+        <v>22091211</v>
+      </c>
+      <c r="G176"/>
+      <c r="H176" t="n">
+        <v>5523000</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="s">
+        <v>35</v>
+      </c>
+      <c r="B177" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C177" t="n">
+        <v>10755</v>
+      </c>
+      <c r="D177"/>
+      <c r="E177" t="n">
+        <v>2739</v>
+      </c>
+      <c r="F177" t="n">
+        <v>28399735</v>
+      </c>
+      <c r="G177"/>
+      <c r="H177" t="n">
+        <v>7283374</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="s">
+        <v>35</v>
+      </c>
+      <c r="B178" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C178" t="n">
+        <v>8607</v>
+      </c>
+      <c r="D178"/>
+      <c r="E178" t="n">
+        <v>2226</v>
+      </c>
+      <c r="F178" t="n">
+        <v>21984423</v>
+      </c>
+      <c r="G178"/>
+      <c r="H178" t="n">
+        <v>5807522</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="s">
+        <v>35</v>
+      </c>
+      <c r="B179" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C179" t="n">
+        <v>9670</v>
+      </c>
+      <c r="D179"/>
+      <c r="E179" t="n">
+        <v>2352</v>
+      </c>
+      <c r="F179" t="n">
+        <v>27963598</v>
+      </c>
+      <c r="G179"/>
+      <c r="H179" t="n">
+        <v>6725843</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="s">
+        <v>35</v>
+      </c>
+      <c r="B180" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C180" t="n">
+        <v>10723</v>
+      </c>
+      <c r="D180"/>
+      <c r="E180" t="n">
+        <v>2681</v>
+      </c>
+      <c r="F180" t="n">
+        <v>32245006</v>
+      </c>
+      <c r="G180"/>
+      <c r="H180" t="n">
+        <v>8061252</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="s">
+        <v>35</v>
+      </c>
+      <c r="B181" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C181" t="n">
+        <v>11073</v>
+      </c>
+      <c r="D181"/>
+      <c r="E181" t="n">
+        <v>2768</v>
+      </c>
+      <c r="F181" t="n">
+        <v>35816654</v>
+      </c>
+      <c r="G181"/>
+      <c r="H181" t="n">
+        <v>8954160</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="s">
+        <v>35</v>
+      </c>
+      <c r="B182" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C182" t="n">
+        <v>10275</v>
+      </c>
+      <c r="D182"/>
+      <c r="E182"/>
+      <c r="F182" t="n">
+        <v>36596063</v>
+      </c>
+      <c r="G182"/>
+      <c r="H182"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="s">
+        <v>36</v>
+      </c>
+      <c r="B183" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C183" t="n">
+        <v>741184</v>
+      </c>
+      <c r="D183"/>
+      <c r="E183" t="n">
+        <v>185296</v>
+      </c>
+      <c r="F183" t="n">
+        <v>4314408732</v>
+      </c>
+      <c r="G183"/>
+      <c r="H183" t="n">
+        <v>1078604000</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="s">
+        <v>36</v>
+      </c>
+      <c r="B184" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C184"/>
+      <c r="D184"/>
+      <c r="E184" t="n">
+        <v>219500</v>
+      </c>
+      <c r="F184"/>
+      <c r="G184"/>
+      <c r="H184" t="n">
+        <v>1308220035</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>